<commit_message>
Agrega modo oscuro/claro, corrige treemap de clientes y actualiza datos de ventas y pipeline
- Toggle de tema claro/oscuro persistente (localStorage) con soporte en toda la app
- Corrige nombres truncados/cortados en el treemap de Top 5 Clientes
- Actualiza márgenes comerciales en ventas.json según Excel
- Regenera pipeline.json desde la pestaña PIPELINE actualizada de BASE COLOMBIA-.xlsx

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/BASE COLOMBIA-.xlsx
+++ b/BASE COLOMBIA-.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\vrodriguez\Desktop\DIRECTORIO CO\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D07457BD-2971-461D-8601-2323DE6DD470}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DD121436-34C1-4C94-8B87-DF5DEF31AB67}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="VENTAS" sheetId="5" r:id="rId1"/>
@@ -738,7 +738,7 @@
     <xf numFmtId="9" fontId="5" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="43" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="58">
+  <cellXfs count="53">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -876,25 +876,10 @@
     </xf>
     <xf numFmtId="166" fontId="7" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="1" applyFont="1"/>
-    <xf numFmtId="9" fontId="3" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="3" fontId="3" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="165" fontId="4" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="165" fontId="3" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="165" fontId="4" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="3" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="4" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -1220,7 +1205,7 @@
         <v>697232.96000000008</v>
       </c>
       <c r="I2" s="50">
-        <v>0.18</v>
+        <v>0.2</v>
       </c>
       <c r="J2" t="s">
         <v>167</v>
@@ -1231,7 +1216,7 @@
     </row>
     <row r="3" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A3">
-        <v>2023</v>
+        <v>2024</v>
       </c>
       <c r="B3" s="43">
         <v>45407</v>
@@ -1255,7 +1240,7 @@
         <v>48000</v>
       </c>
       <c r="I3" s="50">
-        <v>0.18</v>
+        <v>0.2</v>
       </c>
       <c r="J3" t="s">
         <v>79</v>
@@ -1266,7 +1251,7 @@
     </row>
     <row r="4" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A4">
-        <v>2023</v>
+        <v>2024</v>
       </c>
       <c r="B4" s="43">
         <v>45407</v>
@@ -1290,7 +1275,7 @@
         <v>39900</v>
       </c>
       <c r="I4" s="50">
-        <v>0.18</v>
+        <v>0.2</v>
       </c>
       <c r="J4" t="s">
         <v>79</v>
@@ -1325,7 +1310,7 @@
         <v>5167633.9000000004</v>
       </c>
       <c r="I5" s="50">
-        <v>0.18</v>
+        <v>0.2</v>
       </c>
       <c r="J5" t="s">
         <v>70</v>
@@ -1360,7 +1345,7 @@
         <v>149637</v>
       </c>
       <c r="I6" s="50">
-        <v>0.18</v>
+        <v>0.17</v>
       </c>
       <c r="J6" t="s">
         <v>70</v>
@@ -1395,7 +1380,7 @@
         <v>261514.72</v>
       </c>
       <c r="I7" s="50">
-        <v>0.18</v>
+        <v>0.17</v>
       </c>
       <c r="J7" t="s">
         <v>70</v>
@@ -1430,7 +1415,7 @@
         <v>130209.7</v>
       </c>
       <c r="I8" s="50">
-        <v>0.18</v>
+        <v>0.17</v>
       </c>
       <c r="J8" t="s">
         <v>167</v>
@@ -1780,7 +1765,7 @@
         <v>92832</v>
       </c>
       <c r="I18" s="50">
-        <v>0.18</v>
+        <v>0.17</v>
       </c>
       <c r="J18" t="s">
         <v>70</v>
@@ -1815,7 +1800,7 @@
         <v>749045</v>
       </c>
       <c r="I19" s="50">
-        <v>0.18</v>
+        <v>0.17</v>
       </c>
       <c r="J19" t="s">
         <v>70</v>
@@ -1996,7 +1981,7 @@
       <c r="G3" s="35">
         <v>1</v>
       </c>
-      <c r="H3" s="51">
+      <c r="H3" s="11">
         <v>0.05</v>
       </c>
       <c r="I3" s="8" t="s">
@@ -2142,7 +2127,7 @@
       <c r="M6" s="8">
         <v>2026</v>
       </c>
-      <c r="N6" s="55" t="s">
+      <c r="N6" s="51" t="s">
         <v>174</v>
       </c>
     </row>
@@ -2421,7 +2406,7 @@
       <c r="G13" s="12">
         <v>9</v>
       </c>
-      <c r="H13" s="51">
+      <c r="H13" s="11">
         <v>0.05</v>
       </c>
       <c r="I13" s="8" t="s">
@@ -2463,7 +2448,7 @@
       <c r="G14" s="12">
         <v>10</v>
       </c>
-      <c r="H14" s="51">
+      <c r="H14" s="11">
         <v>0.6</v>
       </c>
       <c r="I14" s="8" t="s">
@@ -2502,10 +2487,10 @@
       <c r="F15" s="11">
         <v>0.18</v>
       </c>
-      <c r="G15" s="52">
+      <c r="G15" s="12">
         <v>10</v>
       </c>
-      <c r="H15" s="51">
+      <c r="H15" s="11">
         <v>0.4</v>
       </c>
       <c r="I15" s="8" t="s">
@@ -2544,7 +2529,7 @@
       <c r="F16" s="11">
         <v>0.18</v>
       </c>
-      <c r="G16" s="52">
+      <c r="G16" s="12">
         <v>9</v>
       </c>
       <c r="H16" s="11">
@@ -2671,7 +2656,7 @@
       <c r="G19" s="12">
         <v>10</v>
       </c>
-      <c r="H19" s="51">
+      <c r="H19" s="11">
         <v>0.05</v>
       </c>
       <c r="I19" s="8" t="s">
@@ -2950,17 +2935,17 @@
       <c r="C26" s="9" t="s">
         <v>66</v>
       </c>
-      <c r="D26" s="57"/>
-      <c r="E26" s="54">
+      <c r="D26" s="9"/>
+      <c r="E26" s="10">
         <v>12000000</v>
       </c>
       <c r="F26" s="11">
         <v>0.18</v>
       </c>
-      <c r="G26" s="52">
+      <c r="G26" s="12">
         <v>3</v>
       </c>
-      <c r="H26" s="51">
+      <c r="H26" s="11">
         <v>0.05</v>
       </c>
       <c r="I26" s="8" t="s">
@@ -2990,7 +2975,7 @@
         <v>91</v>
       </c>
       <c r="D27" s="14"/>
-      <c r="E27" s="53">
+      <c r="E27" s="15">
         <v>150000</v>
       </c>
       <c r="F27" s="11">
@@ -3029,7 +3014,7 @@
         <v>104</v>
       </c>
       <c r="D28" s="14"/>
-      <c r="E28" s="54">
+      <c r="E28" s="10">
         <v>250000</v>
       </c>
       <c r="F28" s="11">
@@ -3038,7 +3023,7 @@
       <c r="G28" s="12">
         <v>2</v>
       </c>
-      <c r="H28" s="51">
+      <c r="H28" s="11">
         <v>0.05</v>
       </c>
       <c r="I28" s="8" t="s">
@@ -3096,7 +3081,7 @@
         <v>2027</v>
       </c>
     </row>
-    <row r="30" spans="1:24" ht="27" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:24" ht="27" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A30" s="8" t="s">
         <v>145</v>
       </c>
@@ -3107,7 +3092,7 @@
         <v>101</v>
       </c>
       <c r="D30" s="14"/>
-      <c r="E30" s="54">
+      <c r="E30" s="10">
         <v>100000</v>
       </c>
       <c r="F30" s="11">
@@ -3146,7 +3131,7 @@
         <v>149</v>
       </c>
       <c r="D31" s="19"/>
-      <c r="E31" s="56">
+      <c r="E31" s="52">
         <f>70*600</f>
         <v>42000</v>
       </c>
@@ -3186,7 +3171,7 @@
         <v>66</v>
       </c>
       <c r="D32" s="24"/>
-      <c r="E32" s="53">
+      <c r="E32" s="15">
         <v>2000000</v>
       </c>
       <c r="F32" s="11">

</xml_diff>

<commit_message>
Pipeline: agrega tab Diversificación NO AGRO entre Forecast y Clientes
Reordena los tabs internos (Resumen → Forecast → Diversificación →
Clientes por etapa) y crea Diversificación con selector 2026/2027,
KPIs de pipeline NO AGRO activo/ponderado y participación, barras de
sector y madurez, y tabla ejecutiva de oportunidades — todo con el
mismo lenguaje visual de Resumen/Forecast. Regenera data/pipeline.json
desde la última BASE COLOMBIA-.xlsx (columna AGRO/NO AGRO actualizada).
</commit_message>
<xml_diff>
--- a/BASE COLOMBIA-.xlsx
+++ b/BASE COLOMBIA-.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\vrodriguez\Desktop\DIRECTORIO CO\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DD121436-34C1-4C94-8B87-DF5DEF31AB67}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8289539A-4EF5-455E-AE2C-A18E0C3ED459}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="VENTAS" sheetId="5" r:id="rId1"/>
@@ -738,7 +738,7 @@
     <xf numFmtId="9" fontId="5" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="43" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="53">
+  <cellXfs count="48">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -787,18 +787,6 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="9" fontId="3" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="3" fontId="3" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -862,9 +850,6 @@
     <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -879,8 +864,8 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="165" fontId="4" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="3">
@@ -1135,20 +1120,22 @@
   <dimension ref="A1:K24"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="13.2" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="2" max="2" width="11.5546875" style="43"/>
+    <col min="2" max="2" width="11.5546875" style="39"/>
     <col min="4" max="4" width="33.21875" customWidth="1"/>
-    <col min="6" max="6" width="13.6640625" customWidth="1"/>
-    <col min="8" max="8" width="22" style="42" customWidth="1"/>
-    <col min="9" max="9" width="16.109375" style="42" customWidth="1"/>
+    <col min="5" max="5" width="0" hidden="1" customWidth="1"/>
+    <col min="6" max="6" width="13.6640625" hidden="1" customWidth="1"/>
+    <col min="7" max="7" width="0" hidden="1" customWidth="1"/>
+    <col min="8" max="8" width="22" style="38" hidden="1" customWidth="1"/>
+    <col min="9" max="9" width="16.109375" style="38" customWidth="1"/>
     <col min="10" max="10" width="16.88671875" customWidth="1"/>
-    <col min="11" max="11" width="63.33203125" style="41" customWidth="1"/>
+    <col min="11" max="11" width="63.33203125" style="37" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="43" t="s">
+      <c r="B1" s="39" t="s">
         <v>1</v>
       </c>
       <c r="C1" t="s">
@@ -1166,16 +1153,16 @@
       <c r="G1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="42" t="s">
+      <c r="H1" s="38" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="49" t="s">
+      <c r="I1" s="44" t="s">
         <v>173</v>
       </c>
       <c r="J1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="41" t="s">
+      <c r="K1" s="37" t="s">
         <v>166</v>
       </c>
     </row>
@@ -1183,7 +1170,7 @@
       <c r="A2">
         <v>2023</v>
       </c>
-      <c r="B2" s="43">
+      <c r="B2" s="39">
         <v>45149</v>
       </c>
       <c r="C2" t="s">
@@ -1201,16 +1188,16 @@
       <c r="G2" t="s">
         <v>16</v>
       </c>
-      <c r="H2" s="42">
+      <c r="H2" s="38">
         <v>697232.96000000008</v>
       </c>
-      <c r="I2" s="50">
+      <c r="I2" s="45">
         <v>0.2</v>
       </c>
       <c r="J2" t="s">
         <v>167</v>
       </c>
-      <c r="K2" s="41" t="s">
+      <c r="K2" s="37" t="s">
         <v>168</v>
       </c>
     </row>
@@ -1218,7 +1205,7 @@
       <c r="A3">
         <v>2024</v>
       </c>
-      <c r="B3" s="43">
+      <c r="B3" s="39">
         <v>45407</v>
       </c>
       <c r="C3" t="s">
@@ -1236,16 +1223,16 @@
       <c r="G3" t="s">
         <v>13</v>
       </c>
-      <c r="H3" s="42">
+      <c r="H3" s="38">
         <v>48000</v>
       </c>
-      <c r="I3" s="50">
+      <c r="I3" s="45">
         <v>0.2</v>
       </c>
       <c r="J3" t="s">
         <v>79</v>
       </c>
-      <c r="K3" s="41" t="s">
+      <c r="K3" s="37" t="s">
         <v>169</v>
       </c>
     </row>
@@ -1253,7 +1240,7 @@
       <c r="A4">
         <v>2024</v>
       </c>
-      <c r="B4" s="43">
+      <c r="B4" s="39">
         <v>45407</v>
       </c>
       <c r="C4" t="s">
@@ -1271,16 +1258,16 @@
       <c r="G4" t="s">
         <v>13</v>
       </c>
-      <c r="H4" s="42">
+      <c r="H4" s="38">
         <v>39900</v>
       </c>
-      <c r="I4" s="50">
+      <c r="I4" s="45">
         <v>0.2</v>
       </c>
       <c r="J4" t="s">
         <v>79</v>
       </c>
-      <c r="K4" s="41" t="s">
+      <c r="K4" s="37" t="s">
         <v>170</v>
       </c>
     </row>
@@ -1288,7 +1275,7 @@
       <c r="A5">
         <v>2024</v>
       </c>
-      <c r="B5" s="43">
+      <c r="B5" s="39">
         <v>45596</v>
       </c>
       <c r="C5" t="s">
@@ -1306,16 +1293,16 @@
       <c r="G5" t="s">
         <v>13</v>
       </c>
-      <c r="H5" s="42">
+      <c r="H5" s="38">
         <v>5167633.9000000004</v>
       </c>
-      <c r="I5" s="50">
+      <c r="I5" s="45">
         <v>0.2</v>
       </c>
       <c r="J5" t="s">
         <v>70</v>
       </c>
-      <c r="K5" s="41" t="s">
+      <c r="K5" s="37" t="s">
         <v>22</v>
       </c>
     </row>
@@ -1323,7 +1310,7 @@
       <c r="A6">
         <v>2025</v>
       </c>
-      <c r="B6" s="43">
+      <c r="B6" s="39">
         <v>45757</v>
       </c>
       <c r="C6" t="s">
@@ -1341,16 +1328,16 @@
       <c r="G6" t="s">
         <v>13</v>
       </c>
-      <c r="H6" s="42">
+      <c r="H6" s="38">
         <v>149637</v>
       </c>
-      <c r="I6" s="50">
+      <c r="I6" s="45">
         <v>0.17</v>
       </c>
       <c r="J6" t="s">
         <v>70</v>
       </c>
-      <c r="K6" s="41" t="s">
+      <c r="K6" s="37" t="s">
         <v>27</v>
       </c>
     </row>
@@ -1358,7 +1345,7 @@
       <c r="A7">
         <v>2025</v>
       </c>
-      <c r="B7" s="43">
+      <c r="B7" s="39">
         <v>45761</v>
       </c>
       <c r="C7" t="s">
@@ -1376,16 +1363,16 @@
       <c r="G7" t="s">
         <v>13</v>
       </c>
-      <c r="H7" s="42">
+      <c r="H7" s="38">
         <v>261514.72</v>
       </c>
-      <c r="I7" s="50">
+      <c r="I7" s="45">
         <v>0.17</v>
       </c>
       <c r="J7" t="s">
         <v>70</v>
       </c>
-      <c r="K7" s="41" t="s">
+      <c r="K7" s="37" t="s">
         <v>27</v>
       </c>
     </row>
@@ -1393,7 +1380,7 @@
       <c r="A8">
         <v>2025</v>
       </c>
-      <c r="B8" s="43">
+      <c r="B8" s="39">
         <v>45796</v>
       </c>
       <c r="C8" t="s">
@@ -1411,16 +1398,16 @@
       <c r="G8" t="s">
         <v>13</v>
       </c>
-      <c r="H8" s="42">
+      <c r="H8" s="38">
         <v>130209.7</v>
       </c>
-      <c r="I8" s="50">
+      <c r="I8" s="45">
         <v>0.17</v>
       </c>
       <c r="J8" t="s">
         <v>167</v>
       </c>
-      <c r="K8" s="41" t="s">
+      <c r="K8" s="37" t="s">
         <v>31</v>
       </c>
     </row>
@@ -1428,7 +1415,7 @@
       <c r="A9">
         <v>2025</v>
       </c>
-      <c r="B9" s="43">
+      <c r="B9" s="39">
         <v>45818</v>
       </c>
       <c r="C9" t="s">
@@ -1446,16 +1433,16 @@
       <c r="G9" t="s">
         <v>38</v>
       </c>
-      <c r="H9" s="42">
+      <c r="H9" s="38">
         <v>1640.08</v>
       </c>
-      <c r="I9" s="50">
+      <c r="I9" s="45">
         <v>0.18</v>
       </c>
       <c r="J9" t="s">
         <v>79</v>
       </c>
-      <c r="K9" s="41" t="s">
+      <c r="K9" s="37" t="s">
         <v>40</v>
       </c>
     </row>
@@ -1463,7 +1450,7 @@
       <c r="A10">
         <v>2025</v>
       </c>
-      <c r="B10" s="43">
+      <c r="B10" s="39">
         <v>45835</v>
       </c>
       <c r="C10" t="s">
@@ -1481,16 +1468,16 @@
       <c r="G10" t="s">
         <v>13</v>
       </c>
-      <c r="H10" s="42">
+      <c r="H10" s="38">
         <v>120684.94</v>
       </c>
-      <c r="I10" s="50">
+      <c r="I10" s="45">
         <v>0.18</v>
       </c>
       <c r="J10" t="s">
         <v>70</v>
       </c>
-      <c r="K10" s="41" t="s">
+      <c r="K10" s="37" t="s">
         <v>33</v>
       </c>
     </row>
@@ -1498,7 +1485,7 @@
       <c r="A11">
         <v>2025</v>
       </c>
-      <c r="B11" s="43">
+      <c r="B11" s="39">
         <v>45841</v>
       </c>
       <c r="C11" t="s">
@@ -1516,16 +1503,16 @@
       <c r="G11" t="s">
         <v>13</v>
       </c>
-      <c r="H11" s="42">
+      <c r="H11" s="38">
         <v>1206011</v>
       </c>
-      <c r="I11" s="50">
+      <c r="I11" s="45">
         <v>0.18</v>
       </c>
       <c r="J11" t="s">
         <v>70</v>
       </c>
-      <c r="K11" s="41" t="s">
+      <c r="K11" s="37" t="s">
         <v>43</v>
       </c>
     </row>
@@ -1533,7 +1520,7 @@
       <c r="A12">
         <v>2025</v>
       </c>
-      <c r="B12" s="43">
+      <c r="B12" s="39">
         <v>45862</v>
       </c>
       <c r="C12" t="s">
@@ -1551,16 +1538,16 @@
       <c r="G12" t="s">
         <v>41</v>
       </c>
-      <c r="H12" s="42">
+      <c r="H12" s="38">
         <v>868</v>
       </c>
-      <c r="I12" s="50">
+      <c r="I12" s="45">
         <v>0.18</v>
       </c>
       <c r="J12" t="s">
         <v>167</v>
       </c>
-      <c r="K12" s="41" t="s">
+      <c r="K12" s="37" t="s">
         <v>42</v>
       </c>
     </row>
@@ -1568,7 +1555,7 @@
       <c r="A13">
         <v>2025</v>
       </c>
-      <c r="B13" s="43">
+      <c r="B13" s="39">
         <v>45881</v>
       </c>
       <c r="C13" t="s">
@@ -1586,16 +1573,16 @@
       <c r="G13" t="s">
         <v>13</v>
       </c>
-      <c r="H13" s="42">
+      <c r="H13" s="38">
         <v>30840</v>
       </c>
-      <c r="I13" s="50">
+      <c r="I13" s="45">
         <v>0.18</v>
       </c>
       <c r="J13" t="s">
         <v>79</v>
       </c>
-      <c r="K13" s="41" t="s">
+      <c r="K13" s="37" t="s">
         <v>36</v>
       </c>
     </row>
@@ -1603,7 +1590,7 @@
       <c r="A14">
         <v>2025</v>
       </c>
-      <c r="B14" s="43">
+      <c r="B14" s="39">
         <v>45960</v>
       </c>
       <c r="C14" t="s">
@@ -1621,16 +1608,16 @@
       <c r="G14" t="s">
         <v>38</v>
       </c>
-      <c r="H14" s="42">
+      <c r="H14" s="38">
         <v>3833.2757499999998</v>
       </c>
-      <c r="I14" s="50">
+      <c r="I14" s="45">
         <v>0.18</v>
       </c>
       <c r="J14" t="s">
         <v>70</v>
       </c>
-      <c r="K14" s="41" t="s">
+      <c r="K14" s="37" t="s">
         <v>39</v>
       </c>
     </row>
@@ -1638,7 +1625,7 @@
       <c r="A15">
         <v>2026</v>
       </c>
-      <c r="B15" s="43">
+      <c r="B15" s="39">
         <v>46041</v>
       </c>
       <c r="C15" t="s">
@@ -1656,16 +1643,16 @@
       <c r="G15" t="s">
         <v>38</v>
       </c>
-      <c r="H15" s="42">
+      <c r="H15" s="38">
         <v>1850</v>
       </c>
-      <c r="I15" s="50">
+      <c r="I15" s="45">
         <v>0.18</v>
       </c>
       <c r="J15" t="s">
         <v>167</v>
       </c>
-      <c r="K15" s="41" t="s">
+      <c r="K15" s="37" t="s">
         <v>49</v>
       </c>
     </row>
@@ -1673,7 +1660,7 @@
       <c r="A16">
         <v>2026</v>
       </c>
-      <c r="B16" s="43">
+      <c r="B16" s="39">
         <v>46041</v>
       </c>
       <c r="C16" t="s">
@@ -1691,16 +1678,16 @@
       <c r="G16" t="s">
         <v>38</v>
       </c>
-      <c r="H16" s="42">
+      <c r="H16" s="38">
         <v>300</v>
       </c>
-      <c r="I16" s="50">
+      <c r="I16" s="45">
         <v>0.18</v>
       </c>
       <c r="J16" t="s">
         <v>167</v>
       </c>
-      <c r="K16" s="41" t="s">
+      <c r="K16" s="37" t="s">
         <v>53</v>
       </c>
     </row>
@@ -1708,7 +1695,7 @@
       <c r="A17">
         <v>2026</v>
       </c>
-      <c r="B17" s="43">
+      <c r="B17" s="39">
         <v>46047</v>
       </c>
       <c r="C17" t="s">
@@ -1726,16 +1713,16 @@
       <c r="G17" t="s">
         <v>38</v>
       </c>
-      <c r="H17" s="42">
+      <c r="H17" s="38">
         <v>1298.6300000000001</v>
       </c>
-      <c r="I17" s="50">
+      <c r="I17" s="45">
         <v>0.18</v>
       </c>
       <c r="J17" t="s">
         <v>167</v>
       </c>
-      <c r="K17" s="41" t="s">
+      <c r="K17" s="37" t="s">
         <v>51</v>
       </c>
     </row>
@@ -1743,7 +1730,7 @@
       <c r="A18">
         <v>2026</v>
       </c>
-      <c r="B18" s="43">
+      <c r="B18" s="39">
         <v>46052</v>
       </c>
       <c r="C18" t="s">
@@ -1761,16 +1748,16 @@
       <c r="G18" t="s">
         <v>48</v>
       </c>
-      <c r="H18" s="42">
+      <c r="H18" s="38">
         <v>92832</v>
       </c>
-      <c r="I18" s="50">
+      <c r="I18" s="45">
         <v>0.17</v>
       </c>
       <c r="J18" t="s">
         <v>70</v>
       </c>
-      <c r="K18" s="41" t="s">
+      <c r="K18" s="37" t="s">
         <v>23</v>
       </c>
     </row>
@@ -1778,7 +1765,7 @@
       <c r="A19">
         <v>2026</v>
       </c>
-      <c r="B19" s="43">
+      <c r="B19" s="39">
         <v>46111</v>
       </c>
       <c r="C19" t="s">
@@ -1796,16 +1783,16 @@
       <c r="G19" t="s">
         <v>38</v>
       </c>
-      <c r="H19" s="42">
+      <c r="H19" s="38">
         <v>749045</v>
       </c>
-      <c r="I19" s="50">
+      <c r="I19" s="45">
         <v>0.17</v>
       </c>
       <c r="J19" t="s">
         <v>70</v>
       </c>
-      <c r="K19" s="41" t="s">
+      <c r="K19" s="37" t="s">
         <v>154</v>
       </c>
     </row>
@@ -1813,7 +1800,7 @@
       <c r="A20">
         <v>2026</v>
       </c>
-      <c r="B20" s="43">
+      <c r="B20" s="39">
         <v>46233</v>
       </c>
       <c r="C20" s="1" t="s">
@@ -1831,16 +1818,16 @@
       <c r="G20" s="1" t="s">
         <v>171</v>
       </c>
-      <c r="H20" s="42">
+      <c r="H20" s="38">
         <v>1239.194476744186</v>
       </c>
-      <c r="I20" s="50">
+      <c r="I20" s="45">
         <v>0.18</v>
       </c>
       <c r="J20" t="s">
         <v>79</v>
       </c>
-      <c r="K20" s="41" t="s">
+      <c r="K20" s="37" t="s">
         <v>122</v>
       </c>
     </row>
@@ -1916,7 +1903,7 @@
         <v>158</v>
       </c>
     </row>
-    <row r="2" spans="1:14" ht="27" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:14" ht="27" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="8" t="s">
         <v>99</v>
       </c>
@@ -1936,7 +1923,7 @@
       <c r="F2" s="11">
         <v>0.18</v>
       </c>
-      <c r="G2" s="35">
+      <c r="G2" s="31">
         <v>3</v>
       </c>
       <c r="H2" s="11">
@@ -1949,7 +1936,7 @@
         <v>68</v>
       </c>
       <c r="K2" s="8" t="s">
-        <v>74</v>
+        <v>69</v>
       </c>
       <c r="L2" s="8" t="s">
         <v>70</v>
@@ -1958,7 +1945,7 @@
         <v>2027</v>
       </c>
     </row>
-    <row r="3" spans="1:14" ht="27" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:14" ht="27" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="8" t="s">
         <v>142</v>
       </c>
@@ -1978,7 +1965,7 @@
       <c r="F3" s="11">
         <v>0.18</v>
       </c>
-      <c r="G3" s="35">
+      <c r="G3" s="31">
         <v>1</v>
       </c>
       <c r="H3" s="11">
@@ -1991,7 +1978,7 @@
         <v>78</v>
       </c>
       <c r="K3" s="8" t="s">
-        <v>69</v>
+        <v>74</v>
       </c>
       <c r="L3" s="8" t="s">
         <v>70</v>
@@ -2000,7 +1987,7 @@
         <v>2027</v>
       </c>
     </row>
-    <row r="4" spans="1:14" ht="27" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:14" ht="27" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="8" t="s">
         <v>71</v>
       </c>
@@ -2021,7 +2008,7 @@
       <c r="F4" s="11">
         <v>0.18</v>
       </c>
-      <c r="G4" s="35">
+      <c r="G4" s="31">
         <v>1</v>
       </c>
       <c r="H4" s="11">
@@ -2053,7 +2040,7 @@
       <c r="C5" s="9" t="s">
         <v>66</v>
       </c>
-      <c r="D5" s="27">
+      <c r="D5" s="23">
         <f>1912997580+1118985120</f>
         <v>3031982700</v>
       </c>
@@ -2119,7 +2106,7 @@
         <v>96</v>
       </c>
       <c r="K6" s="8" t="s">
-        <v>74</v>
+        <v>69</v>
       </c>
       <c r="L6" s="8" t="s">
         <v>70</v>
@@ -2127,7 +2114,7 @@
       <c r="M6" s="8">
         <v>2026</v>
       </c>
-      <c r="N6" s="51" t="s">
+      <c r="N6" s="46" t="s">
         <v>174</v>
       </c>
     </row>
@@ -2206,7 +2193,7 @@
         <v>78</v>
       </c>
       <c r="K8" s="8" t="s">
-        <v>74</v>
+        <v>69</v>
       </c>
       <c r="L8" s="8" t="s">
         <v>70</v>
@@ -2248,7 +2235,7 @@
         <v>78</v>
       </c>
       <c r="K9" s="8" t="s">
-        <v>74</v>
+        <v>69</v>
       </c>
       <c r="L9" s="8" t="s">
         <v>70</v>
@@ -2277,7 +2264,7 @@
       <c r="F10" s="11">
         <v>0.18</v>
       </c>
-      <c r="G10" s="35">
+      <c r="G10" s="31">
         <v>1</v>
       </c>
       <c r="H10" s="11">
@@ -2624,7 +2611,7 @@
         <v>78</v>
       </c>
       <c r="K18" s="8" t="s">
-        <v>69</v>
+        <v>74</v>
       </c>
       <c r="L18" s="8" t="s">
         <v>70</v>
@@ -2748,7 +2735,7 @@
         <v>78</v>
       </c>
       <c r="K21" s="8" t="s">
-        <v>69</v>
+        <v>74</v>
       </c>
       <c r="L21" s="8" t="s">
         <v>79</v>
@@ -2874,7 +2861,7 @@
         <v>78</v>
       </c>
       <c r="K24" s="8" t="s">
-        <v>74</v>
+        <v>69</v>
       </c>
       <c r="L24" s="8" t="s">
         <v>79</v>
@@ -2925,7 +2912,7 @@
         <v>2026</v>
       </c>
     </row>
-    <row r="26" spans="1:24" ht="27" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:24" ht="27" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A26" s="8" t="s">
         <v>86</v>
       </c>
@@ -2955,7 +2942,7 @@
         <v>88</v>
       </c>
       <c r="K26" s="8" t="s">
-        <v>69</v>
+        <v>74</v>
       </c>
       <c r="L26" s="8" t="s">
         <v>70</v>
@@ -3003,7 +2990,7 @@
         <v>2026</v>
       </c>
     </row>
-    <row r="28" spans="1:24" ht="27" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:24" ht="27" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A28" s="8" t="s">
         <v>103</v>
       </c>
@@ -3042,7 +3029,7 @@
         <v>2027</v>
       </c>
     </row>
-    <row r="29" spans="1:24" ht="27" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:24" ht="27" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A29" s="8" t="s">
         <v>103</v>
       </c>
@@ -3059,7 +3046,7 @@
       <c r="F29" s="11">
         <v>0.18</v>
       </c>
-      <c r="G29" s="35">
+      <c r="G29" s="31">
         <v>3</v>
       </c>
       <c r="H29" s="11">
@@ -3072,7 +3059,7 @@
         <v>68</v>
       </c>
       <c r="K29" s="8" t="s">
-        <v>69</v>
+        <v>74</v>
       </c>
       <c r="L29" s="8" t="s">
         <v>79</v>
@@ -3081,7 +3068,7 @@
         <v>2027</v>
       </c>
     </row>
-    <row r="30" spans="1:24" ht="27" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:24" ht="27" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A30" s="8" t="s">
         <v>145</v>
       </c>
@@ -3098,7 +3085,7 @@
       <c r="F30" s="11">
         <v>0.18</v>
       </c>
-      <c r="G30" s="35">
+      <c r="G30" s="31">
         <v>6</v>
       </c>
       <c r="H30" s="11">
@@ -3120,67 +3107,67 @@
         <v>2027</v>
       </c>
     </row>
-    <row r="31" spans="1:24" ht="27" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A31" s="18" t="s">
+    <row r="31" spans="1:24" ht="27" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A31" s="13" t="s">
         <v>147</v>
       </c>
-      <c r="B31" s="18" t="s">
+      <c r="B31" s="13" t="s">
         <v>148</v>
       </c>
-      <c r="C31" s="19" t="s">
+      <c r="C31" s="14" t="s">
         <v>149</v>
       </c>
-      <c r="D31" s="19"/>
-      <c r="E31" s="52">
+      <c r="D31" s="14"/>
+      <c r="E31" s="15">
         <f>70*600</f>
         <v>42000</v>
       </c>
-      <c r="F31" s="20">
-        <v>0.18</v>
-      </c>
-      <c r="G31" s="21">
+      <c r="F31" s="11">
+        <v>0.18</v>
+      </c>
+      <c r="G31" s="12">
         <v>11</v>
       </c>
-      <c r="H31" s="20">
+      <c r="H31" s="11">
         <v>0.2</v>
       </c>
-      <c r="I31" s="22" t="s">
+      <c r="I31" s="8" t="s">
         <v>87</v>
       </c>
-      <c r="J31" s="22" t="s">
+      <c r="J31" s="8" t="s">
         <v>78</v>
       </c>
-      <c r="K31" s="22" t="s">
+      <c r="K31" s="8" t="s">
         <v>69</v>
       </c>
-      <c r="L31" s="22" t="s">
+      <c r="L31" s="18" t="s">
         <v>70</v>
       </c>
       <c r="M31" s="8">
         <v>2026</v>
       </c>
     </row>
-    <row r="32" spans="1:24" ht="27" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A32" s="23" t="s">
+    <row r="32" spans="1:24" ht="27" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A32" s="19" t="s">
         <v>155</v>
       </c>
-      <c r="B32" s="23" t="s">
+      <c r="B32" s="19" t="s">
         <v>156</v>
       </c>
-      <c r="C32" s="24" t="s">
+      <c r="C32" s="20" t="s">
         <v>66</v>
       </c>
-      <c r="D32" s="24"/>
+      <c r="D32" s="20"/>
       <c r="E32" s="15">
         <v>2000000</v>
       </c>
       <c r="F32" s="11">
         <v>0.18</v>
       </c>
-      <c r="G32" s="23">
+      <c r="G32" s="19">
         <v>1</v>
       </c>
-      <c r="H32" s="25">
+      <c r="H32" s="21">
         <v>0.4</v>
       </c>
       <c r="I32" s="8" t="s">
@@ -3192,7 +3179,7 @@
       <c r="K32" s="8" t="s">
         <v>74</v>
       </c>
-      <c r="L32" s="24" t="s">
+      <c r="L32" s="20" t="s">
         <v>70</v>
       </c>
       <c r="M32" s="8">
@@ -3216,11 +3203,6 @@
         <filter val="Negociación"/>
         <filter val="Postpuesto"/>
         <filter val="Prospecto"/>
-      </filters>
-    </filterColumn>
-    <filterColumn colId="12">
-      <filters>
-        <filter val="2026"/>
       </filters>
     </filterColumn>
     <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:M32">
@@ -3244,7 +3226,7 @@
   <sheetFormatPr baseColWidth="10" defaultRowHeight="13.2" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="22.5546875" customWidth="1"/>
-    <col min="2" max="2" width="24.44140625" style="31" customWidth="1"/>
+    <col min="2" max="2" width="24.44140625" style="27" customWidth="1"/>
     <col min="4" max="4" width="20" customWidth="1"/>
     <col min="5" max="5" width="15.6640625" customWidth="1"/>
     <col min="6" max="6" width="15" customWidth="1"/>
@@ -3253,192 +3235,192 @@
   </cols>
   <sheetData>
     <row r="2" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A2" s="26" t="s">
+      <c r="A2" s="22" t="s">
         <v>150</v>
       </c>
-      <c r="B2" s="32"/>
-      <c r="C2" s="26"/>
-      <c r="D2" s="26"/>
+      <c r="B2" s="28"/>
+      <c r="C2" s="22"/>
+      <c r="D2" s="22"/>
     </row>
     <row r="3" spans="1:12" ht="26.4" x14ac:dyDescent="0.25">
-      <c r="A3" s="24" t="s">
+      <c r="A3" s="20" t="s">
         <v>158</v>
       </c>
-      <c r="B3" s="24" t="s">
+      <c r="B3" s="20" t="s">
         <v>159</v>
       </c>
-      <c r="C3" s="24" t="s">
+      <c r="C3" s="20" t="s">
         <v>160</v>
       </c>
-      <c r="D3" s="24" t="s">
+      <c r="D3" s="20" t="s">
         <v>54</v>
       </c>
-      <c r="E3" s="24" t="s">
+      <c r="E3" s="20" t="s">
         <v>62</v>
       </c>
-      <c r="F3" s="24" t="s">
+      <c r="F3" s="20" t="s">
         <v>161</v>
       </c>
-      <c r="G3" s="24" t="s">
+      <c r="G3" s="20" t="s">
         <v>162</v>
       </c>
-      <c r="H3" s="24" t="s">
+      <c r="H3" s="20" t="s">
         <v>163</v>
       </c>
     </row>
     <row r="4" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A4" s="28">
-        <v>2026</v>
-      </c>
-      <c r="B4" s="29">
+      <c r="A4" s="24">
+        <v>2026</v>
+      </c>
+      <c r="B4" s="25">
         <v>46041</v>
       </c>
-      <c r="C4" s="28" t="s">
+      <c r="C4" s="24" t="s">
         <v>46</v>
       </c>
-      <c r="D4" s="28" t="s">
+      <c r="D4" s="24" t="s">
         <v>18</v>
       </c>
-      <c r="E4" s="28" t="s">
+      <c r="E4" s="24" t="s">
         <v>19</v>
       </c>
-      <c r="F4" s="34">
+      <c r="F4" s="30">
         <v>1850</v>
       </c>
-      <c r="G4" s="30">
-        <v>0.18</v>
-      </c>
-      <c r="H4" s="28" t="s">
+      <c r="G4" s="26">
+        <v>0.18</v>
+      </c>
+      <c r="H4" s="24" t="s">
         <v>49</v>
       </c>
     </row>
     <row r="5" spans="1:12" ht="26.4" x14ac:dyDescent="0.25">
-      <c r="A5" s="28">
-        <v>2026</v>
-      </c>
-      <c r="B5" s="29">
+      <c r="A5" s="24">
+        <v>2026</v>
+      </c>
+      <c r="B5" s="25">
         <v>46041</v>
       </c>
-      <c r="C5" s="28" t="s">
+      <c r="C5" s="24" t="s">
         <v>46</v>
       </c>
-      <c r="D5" s="28" t="s">
+      <c r="D5" s="24" t="s">
         <v>52</v>
       </c>
-      <c r="E5" s="28" t="s">
+      <c r="E5" s="24" t="s">
         <v>19</v>
       </c>
-      <c r="F5" s="34">
+      <c r="F5" s="30">
         <v>300</v>
       </c>
-      <c r="G5" s="30">
-        <v>0.18</v>
-      </c>
-      <c r="H5" s="28" t="s">
+      <c r="G5" s="26">
+        <v>0.18</v>
+      </c>
+      <c r="H5" s="24" t="s">
         <v>53</v>
       </c>
     </row>
     <row r="6" spans="1:12" ht="26.4" x14ac:dyDescent="0.25">
-      <c r="A6" s="28">
-        <v>2026</v>
-      </c>
-      <c r="B6" s="29">
+      <c r="A6" s="24">
+        <v>2026</v>
+      </c>
+      <c r="B6" s="25">
         <v>46047</v>
       </c>
-      <c r="C6" s="28" t="s">
+      <c r="C6" s="24" t="s">
         <v>46</v>
       </c>
-      <c r="D6" s="28" t="s">
+      <c r="D6" s="24" t="s">
         <v>50</v>
       </c>
-      <c r="E6" s="28" t="s">
+      <c r="E6" s="24" t="s">
         <v>19</v>
       </c>
-      <c r="F6" s="34">
+      <c r="F6" s="30">
         <v>1298.6300000000001</v>
       </c>
-      <c r="G6" s="30">
-        <v>0.18</v>
-      </c>
-      <c r="H6" s="28" t="s">
+      <c r="G6" s="26">
+        <v>0.18</v>
+      </c>
+      <c r="H6" s="24" t="s">
         <v>51</v>
       </c>
     </row>
     <row r="7" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A7" s="28">
-        <v>2026</v>
-      </c>
-      <c r="B7" s="29">
+      <c r="A7" s="24">
+        <v>2026</v>
+      </c>
+      <c r="B7" s="25">
         <v>46052</v>
       </c>
-      <c r="C7" s="28" t="s">
+      <c r="C7" s="24" t="s">
         <v>46</v>
       </c>
-      <c r="D7" s="28" t="s">
+      <c r="D7" s="24" t="s">
         <v>10</v>
       </c>
-      <c r="E7" s="28" t="s">
+      <c r="E7" s="24" t="s">
         <v>12</v>
       </c>
-      <c r="F7" s="34">
+      <c r="F7" s="30">
         <v>92832</v>
       </c>
-      <c r="G7" s="30">
-        <v>0.18</v>
-      </c>
-      <c r="H7" s="28" t="s">
+      <c r="G7" s="26">
+        <v>0.18</v>
+      </c>
+      <c r="H7" s="24" t="s">
         <v>23</v>
       </c>
     </row>
     <row r="8" spans="1:12" ht="26.4" x14ac:dyDescent="0.25">
-      <c r="A8" s="28">
-        <v>2026</v>
-      </c>
-      <c r="B8" s="29">
+      <c r="A8" s="24">
+        <v>2026</v>
+      </c>
+      <c r="B8" s="25">
         <v>46111</v>
       </c>
-      <c r="C8" s="28" t="s">
+      <c r="C8" s="24" t="s">
         <v>44</v>
       </c>
-      <c r="D8" s="28" t="s">
+      <c r="D8" s="24" t="s">
         <v>45</v>
       </c>
-      <c r="E8" s="28" t="s">
+      <c r="E8" s="24" t="s">
         <v>12</v>
       </c>
-      <c r="F8" s="34">
+      <c r="F8" s="30">
         <v>749045</v>
       </c>
-      <c r="G8" s="30">
-        <v>0.18</v>
-      </c>
-      <c r="H8" s="28" t="s">
+      <c r="G8" s="26">
+        <v>0.18</v>
+      </c>
+      <c r="H8" s="24" t="s">
         <v>154</v>
       </c>
     </row>
     <row r="9" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A9" s="45">
-        <v>2026</v>
-      </c>
-      <c r="B9" s="44">
+      <c r="A9" s="40">
+        <v>2026</v>
+      </c>
+      <c r="B9" s="47">
         <v>46237</v>
       </c>
-      <c r="C9" s="45" t="s">
+      <c r="C9" s="40" t="s">
         <v>34</v>
       </c>
-      <c r="D9" s="45" t="s">
+      <c r="D9" s="40" t="s">
         <v>32</v>
       </c>
-      <c r="E9" s="45" t="s">
+      <c r="E9" s="40" t="s">
         <v>12</v>
       </c>
-      <c r="F9" s="34">
+      <c r="F9" s="30">
         <v>1239.194476744186</v>
       </c>
-      <c r="G9" s="30">
-        <v>0.18</v>
-      </c>
-      <c r="H9" s="45" t="s">
+      <c r="G9" s="26">
+        <v>0.18</v>
+      </c>
+      <c r="H9" s="40" t="s">
         <v>122</v>
       </c>
     </row>
@@ -3495,7 +3477,7 @@
       <c r="C15" s="9" t="s">
         <v>66</v>
       </c>
-      <c r="D15" s="27">
+      <c r="D15" s="23">
         <v>3031982700</v>
       </c>
       <c r="E15" s="10">
@@ -3545,7 +3527,7 @@
       <c r="G16" s="12">
         <v>9</v>
       </c>
-      <c r="H16" s="36">
+      <c r="H16" s="32">
         <v>0.2</v>
       </c>
       <c r="I16" s="8" t="s">
@@ -3600,26 +3582,26 @@
       </c>
     </row>
     <row r="18" spans="1:12" ht="26.4" x14ac:dyDescent="0.25">
-      <c r="A18" s="23" t="s">
+      <c r="A18" s="19" t="s">
         <v>155</v>
       </c>
-      <c r="B18" s="23" t="s">
+      <c r="B18" s="19" t="s">
         <v>156</v>
       </c>
-      <c r="C18" s="24" t="s">
+      <c r="C18" s="20" t="s">
         <v>66</v>
       </c>
-      <c r="D18" s="24"/>
-      <c r="E18" s="40" t="s">
+      <c r="D18" s="20"/>
+      <c r="E18" s="36" t="s">
         <v>157</v>
       </c>
       <c r="F18" s="11">
         <v>0.18</v>
       </c>
-      <c r="G18" s="23">
+      <c r="G18" s="19">
         <v>10</v>
       </c>
-      <c r="H18" s="25">
+      <c r="H18" s="21">
         <v>0.4</v>
       </c>
       <c r="I18" s="8" t="s">
@@ -3691,7 +3673,7 @@
       <c r="C23" s="9" t="s">
         <v>66</v>
       </c>
-      <c r="D23" s="27">
+      <c r="D23" s="23">
         <v>3031982700</v>
       </c>
       <c r="E23" s="10">
@@ -3806,7 +3788,7 @@
         <v>91</v>
       </c>
       <c r="D26" s="14"/>
-      <c r="E26" s="38">
+      <c r="E26" s="34">
         <v>150000</v>
       </c>
       <c r="F26" s="11">
@@ -3842,7 +3824,7 @@
         <v>104</v>
       </c>
       <c r="D27" s="14"/>
-      <c r="E27" s="39">
+      <c r="E27" s="35">
         <v>80000</v>
       </c>
       <c r="F27" s="11">
@@ -3886,7 +3868,7 @@
       <c r="F28" s="11">
         <v>0.18</v>
       </c>
-      <c r="G28" s="37">
+      <c r="G28" s="33">
         <v>9</v>
       </c>
       <c r="H28" s="11">
@@ -3927,7 +3909,7 @@
       <c r="G29" s="12">
         <v>9</v>
       </c>
-      <c r="H29" s="36">
+      <c r="H29" s="32">
         <v>0.2</v>
       </c>
       <c r="I29" s="8" t="s">
@@ -4096,26 +4078,26 @@
       </c>
     </row>
     <row r="34" spans="1:12" ht="26.4" x14ac:dyDescent="0.25">
-      <c r="A34" s="23" t="s">
+      <c r="A34" s="19" t="s">
         <v>155</v>
       </c>
-      <c r="B34" s="23" t="s">
+      <c r="B34" s="19" t="s">
         <v>156</v>
       </c>
-      <c r="C34" s="24" t="s">
+      <c r="C34" s="20" t="s">
         <v>66</v>
       </c>
-      <c r="D34" s="24"/>
-      <c r="E34" s="40" t="s">
+      <c r="D34" s="20"/>
+      <c r="E34" s="36" t="s">
         <v>157</v>
       </c>
       <c r="F34" s="11">
         <v>0.18</v>
       </c>
-      <c r="G34" s="23">
+      <c r="G34" s="19">
         <v>10</v>
       </c>
-      <c r="H34" s="25">
+      <c r="H34" s="21">
         <v>0.4</v>
       </c>
       <c r="I34" s="8" t="s">
@@ -4181,11 +4163,11 @@
       <c r="A39" s="8" t="s">
         <v>64</v>
       </c>
-      <c r="B39" s="46" t="s">
+      <c r="B39" s="41" t="s">
         <v>172</v>
       </c>
-      <c r="C39" s="47"/>
-      <c r="D39" s="33">
+      <c r="C39" s="42"/>
+      <c r="D39" s="29">
         <v>122366.6275</v>
       </c>
       <c r="E39" s="11">
@@ -4197,7 +4179,7 @@
       <c r="G39" s="11">
         <v>0.8</v>
       </c>
-      <c r="H39" s="48" t="s">
+      <c r="H39" s="43" t="s">
         <v>67</v>
       </c>
       <c r="I39" s="8" t="s">

</xml_diff>

<commit_message>
Pipeline/Organigrama: extiende iconos con placa 3D, sincroniza datos 2027
- Regenera data/pipeline.json desde la última BASE COLOMBIA-.xlsx: el
  selector 2027 de Diversificación queda al día (GREENLAND y GRUPO 13
  pasan a estado Prospecto, según la fuente).
- Pipeline: aplica el mismo lenguaje de placa+sombra+hover ya usado en
  KPIs/embudo a los iconos líder de títulos de card (Embudo, Forecast,
  Diversificación, Resumen mensual) y a las cards de etapa de Forecast.
- Organigrama: mismo tratamiento para el icono del hero y el estado
  vacío de "Costo de empresa", igualando el resto de la app.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/BASE COLOMBIA-.xlsx
+++ b/BASE COLOMBIA-.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\vrodriguez\Desktop\DIRECTORIO CO\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8289539A-4EF5-455E-AE2C-A18E0C3ED459}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B3DF2D0E-DB5C-414D-BDCE-9F22E0C46B7C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -570,11 +570,12 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="4">
+  <numFmts count="5">
     <numFmt numFmtId="43" formatCode="_-* #,##0.00_-;\-* #,##0.00_-;_-* &quot;-&quot;??_-;_-@_-"/>
     <numFmt numFmtId="164" formatCode="[$$]#,##0"/>
     <numFmt numFmtId="165" formatCode="[$$]#,##0.00"/>
     <numFmt numFmtId="166" formatCode="[$$-540A]#,##0.00"/>
+    <numFmt numFmtId="167" formatCode="[$$]#,##0.00" x16r2:formatCode16="[$$-sn-Latn-ZW]#,##0.00"/>
   </numFmts>
   <fonts count="10" x14ac:knownFonts="1">
     <font>
@@ -738,7 +739,7 @@
     <xf numFmtId="9" fontId="5" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="43" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="48">
+  <cellXfs count="50">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -867,6 +868,8 @@
     <xf numFmtId="14" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="167" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="Millares 12" xfId="2" xr:uid="{938D1D8F-423C-46A2-80B6-3BA5B9FE60E1}"/>
@@ -1848,13 +1851,13 @@
   <sheetPr filterMode="1">
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
-  <dimension ref="A1:X32"/>
+  <dimension ref="A1:X38"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="12.6640625" defaultRowHeight="27" customHeight="1" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="40.77734375" customWidth="1"/>
     <col min="2" max="2" width="25.33203125" customWidth="1"/>
     <col min="3" max="3" width="12.6640625" customWidth="1"/>
-    <col min="4" max="4" width="15.6640625" customWidth="1"/>
+    <col min="4" max="4" width="15.6640625" hidden="1" customWidth="1"/>
     <col min="5" max="5" width="17" customWidth="1"/>
     <col min="6" max="6" width="12.6640625" customWidth="1"/>
     <col min="7" max="7" width="15.6640625" customWidth="1"/>
@@ -1930,7 +1933,7 @@
         <v>0.4</v>
       </c>
       <c r="I2" s="8" t="s">
-        <v>102</v>
+        <v>87</v>
       </c>
       <c r="J2" s="8" t="s">
         <v>68</v>
@@ -1972,7 +1975,7 @@
         <v>0.05</v>
       </c>
       <c r="I3" s="8" t="s">
-        <v>102</v>
+        <v>87</v>
       </c>
       <c r="J3" s="8" t="s">
         <v>78</v>
@@ -2030,7 +2033,7 @@
         <v>2027</v>
       </c>
     </row>
-    <row r="5" spans="1:14" ht="27" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:14" ht="27" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="8" t="s">
         <v>64</v>
       </c>
@@ -2073,7 +2076,7 @@
         <v>2026</v>
       </c>
     </row>
-    <row r="6" spans="1:14" ht="27" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:14" ht="27" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="8" t="s">
         <v>143</v>
       </c>
@@ -2160,7 +2163,7 @@
         <v>2026</v>
       </c>
     </row>
-    <row r="8" spans="1:14" ht="27" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:14" ht="27" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="8" t="s">
         <v>119</v>
       </c>
@@ -2202,7 +2205,7 @@
         <v>2026</v>
       </c>
     </row>
-    <row r="9" spans="1:14" ht="27" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:14" ht="27" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="8" t="s">
         <v>124</v>
       </c>
@@ -2286,7 +2289,7 @@
         <v>2027</v>
       </c>
     </row>
-    <row r="11" spans="1:14" ht="27" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:14" ht="27" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" s="8" t="s">
         <v>89</v>
       </c>
@@ -2370,7 +2373,7 @@
         <v>2026</v>
       </c>
     </row>
-    <row r="13" spans="1:14" ht="27" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:14" ht="27" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13" s="8" t="s">
         <v>108</v>
       </c>
@@ -2412,7 +2415,7 @@
         <v>2026</v>
       </c>
     </row>
-    <row r="14" spans="1:14" ht="27" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:14" ht="27" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A14" s="8" t="s">
         <v>83</v>
       </c>
@@ -2454,7 +2457,7 @@
         <v>2026</v>
       </c>
     </row>
-    <row r="15" spans="1:14" ht="27" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:14" ht="27" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A15" s="8" t="s">
         <v>116</v>
       </c>
@@ -2496,7 +2499,7 @@
         <v>2026</v>
       </c>
     </row>
-    <row r="16" spans="1:14" ht="27" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:14" ht="27" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A16" s="13" t="s">
         <v>105</v>
       </c>
@@ -2578,7 +2581,7 @@
         <v>2026</v>
       </c>
     </row>
-    <row r="18" spans="1:24" ht="27" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:24" ht="27" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A18" s="8" t="s">
         <v>133</v>
       </c>
@@ -2620,7 +2623,7 @@
         <v>2026</v>
       </c>
     </row>
-    <row r="19" spans="1:24" ht="27" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:24" ht="27" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A19" s="8" t="s">
         <v>80</v>
       </c>
@@ -2702,7 +2705,7 @@
         <v>2026</v>
       </c>
     </row>
-    <row r="21" spans="1:24" ht="27" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:24" ht="27" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A21" s="8" t="s">
         <v>127</v>
       </c>
@@ -2828,7 +2831,7 @@
         <v>2026</v>
       </c>
     </row>
-    <row r="24" spans="1:24" ht="27" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:24" ht="27" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A24" s="8" t="s">
         <v>75</v>
       </c>
@@ -2870,7 +2873,7 @@
         <v>2026</v>
       </c>
     </row>
-    <row r="25" spans="1:24" ht="27" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:24" ht="27" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A25" s="13" t="s">
         <v>131</v>
       </c>
@@ -2951,7 +2954,7 @@
         <v>2027</v>
       </c>
     </row>
-    <row r="27" spans="1:24" ht="27" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:24" ht="27" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A27" s="13" t="s">
         <v>97</v>
       </c>
@@ -3068,7 +3071,7 @@
         <v>2027</v>
       </c>
     </row>
-    <row r="30" spans="1:24" ht="27" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:24" ht="27" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A30" s="8" t="s">
         <v>145</v>
       </c>
@@ -3107,7 +3110,7 @@
         <v>2027</v>
       </c>
     </row>
-    <row r="31" spans="1:24" ht="27" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:24" ht="27" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A31" s="13" t="s">
         <v>147</v>
       </c>
@@ -3193,6 +3196,16 @@
       <c r="V32" s="2"/>
       <c r="W32" s="2"/>
       <c r="X32" s="2"/>
+    </row>
+    <row r="36" spans="4:5" ht="27" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="D36" s="48"/>
+      <c r="E36" s="48"/>
+    </row>
+    <row r="37" spans="4:5" ht="27" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="D37" s="49"/>
+    </row>
+    <row r="38" spans="4:5" ht="27" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="D38" s="48"/>
     </row>
   </sheetData>
   <autoFilter ref="A1:M32" xr:uid="{00000000-0001-0000-0100-000000000000}">
@@ -3203,6 +3216,11 @@
         <filter val="Negociación"/>
         <filter val="Postpuesto"/>
         <filter val="Prospecto"/>
+      </filters>
+    </filterColumn>
+    <filterColumn colId="12">
+      <filters>
+        <filter val="2027"/>
       </filters>
     </filterColumn>
     <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:M32">

</xml_diff>